<commit_message>
Drop tail and chafing sleeve specs from RFQs, keep quantities
No tail certificate is available; specs will be requested by e-mail
(same as previous supply or compatible with the 42mm mooring rope).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PvWX4UZieeRNPMMhCxEuz6
</commit_message>
<xml_diff>
--- a/rfq/IOB_RFQ_to_DSR_-_Chafing_Sleeve.xlsx
+++ b/rfq/IOB_RFQ_to_DSR_-_Chafing_Sleeve.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
   <si>
     <t xml:space="preserve">REQUEST FOR QUOTATION</t>
   </si>
@@ -143,25 +143,11 @@
     <t xml:space="preserve">AEOLUS</t>
   </si>
   <si>
-    <t xml:space="preserve">Chafing sleeve (chafe guard)
+    <t xml:space="preserve">Chafing sleeve
 for Ø42 mm mooring rope</t>
   </si>
   <si>
-    <t xml:space="preserve">DSR or equivalent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For rope Ref. Cert. UMC1151-1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Mooring line accessory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">To fit Ø42 mm UHMWPE (Dyneema) 12-strand mooring rope,
-MBL 127 TON (DSR SUPERMAX, Cert. UMC1151-1)
-Type: tubular abrasion sleeve, slides over rope / eye
-Inner dia.: to suit Ø42 mm rope - supplier to confirm
-Length: please quote standard length (e.g. 1.5 m / 2.0 m)
-Material: supplier to propose (polyester / UHMWPE)</t>
   </si>
   <si>
     <t xml:space="preserve">PCS</t>
@@ -1015,7 +1001,7 @@
       <c r="M13" s="8"/>
       <c r="N13" s="8"/>
     </row>
-    <row r="14" customFormat="false" ht="82.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="n">
         <v>1</v>
       </c>
@@ -1025,23 +1011,17 @@
       <c r="C14" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>43</v>
-      </c>
+      <c r="G14" s="11"/>
       <c r="H14" s="9" t="n">
         <v>10</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="J14" s="12"/>
       <c r="K14" s="13" t="str">
@@ -1052,33 +1032,27 @@
       <c r="M14" s="14"/>
       <c r="N14" s="15"/>
     </row>
-    <row r="15" customFormat="false" ht="82.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E15" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>43</v>
-      </c>
+      <c r="G15" s="11"/>
       <c r="H15" s="9" t="n">
         <v>6</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="J15" s="12"/>
       <c r="K15" s="13" t="str">
@@ -1116,7 +1090,7 @@
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
       <c r="J17" s="17" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="K17" s="18" t="n">
         <f aca="false">SUM(K14:K15)</f>
@@ -1144,7 +1118,7 @@
     </row>
     <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -1162,7 +1136,7 @@
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1228,7 +1202,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1236,16 +1210,16 @@
         <v>24</v>
       </c>
       <c r="B3" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="21" t="s">
         <v>50</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1253,13 +1227,13 @@
         <v>38</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E4" s="23" t="n">
         <f aca="false">COUNTIF(RFQ!$B$14:$B$15,A4)</f>
@@ -1268,16 +1242,16 @@
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B5" s="23" t="n">
         <v>9958303</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E5" s="23" t="n">
         <f aca="false">COUNTIF(RFQ!$B$14:$B$15,A5)</f>
@@ -1293,7 +1267,7 @@
     </row>
     <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>